<commit_message>
Fix Westford engineer's surname: Starrat -> Starratt
Transcription error; confirmed against Westford's Town Manager email. One xlsx
cell (Contacts!B29, by Jim in LibreOffice) drives the witness line + Westford
tag; two photo captions fixed in photo_manifest.csv. Rebuilt: 66 pages, verify
PASS, witness line reads 'Paul Starratt (Westford)'.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Acton Bounds.xlsx
+++ b/Acton Bounds.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId3"/>
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Monuments!$N$1:$N$993</definedName>
-    <definedName function="false" hidden="false" name="CornersForMapping" vbProcedure="false">#REF!</definedName>
+    <definedName function="false" hidden="false" name="CornersForMapping" vbProcedure="false">#ref!</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -1248,7 +1248,7 @@
     <t xml:space="preserve">Paul</t>
   </si>
   <si>
-    <t xml:space="preserve">Starrat</t>
+    <t xml:space="preserve">Starratt</t>
   </si>
   <si>
     <t xml:space="preserve">Richard</t>

</xml_diff>